<commit_message>
chore: update UI translations (IT, DE)
</commit_message>
<xml_diff>
--- a/web-console-ui-translations/dist/translations.xlsx
+++ b/web-console-ui-translations/dist/translations.xlsx
@@ -834,7 +834,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>host</t>
+          <t>ospite</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Arbeitsbereich Dateien</t>
+          <t>Arbeitsbereich-Dateien</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Apprezziamo il fatto che abbia dedicato del tempo a darci un feedback e lavoreremo per
+          <t>Apprezziamo il fatto che abbia dedicato del tempo a fornirci un feedback e lavoreremo per
           risolvere i problemi che ha elencato.</t>
         </is>
       </c>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Invia</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Consenti l'accesso degli ospiti allo spazio di lavoro $t(assets)</t>
+          <t>Consenti l'accesso ospite allo spazio di lavoro $t(assets)</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>No $t(assets) $t(selected)@</t>
+          <t>No $t(assets) $t(selected)</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>In attesa della guida...</t>
+          <t>In attesa dell'host...</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Desidera mantenere la SuperFreeze come risorsa?</t>
+          <t>Vuole mantenere il SuperFreeze come asset?</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Wenn diese Funktion aktiviert ist, können Gäste an der Besprechung teilnehmen, ohne dass ein Host anwesend ist.</t>
+          <t>Wenn diese Funktion aktiviert ist, können Gäste an einem Meeting teilnehmen, ohne dass ein Host anwesend ist.</t>
         </is>
       </c>
     </row>
@@ -5897,12 +5897,12 @@
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Quando è abilitato, gli Host e gli Ospiti possono utilizzare le funzioni relative allo storage, compresa la Libreria delle risorse.</t>
+          <t>Quando è abilitato, gli Host e gli Ospiti possono utilizzare le funzioni relative all'archiviazione, compresa la Libreria di risorse.</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Wenn diese Funktion aktiviert ist, können Hosts und Gäste speicherbezogene Funktionen, einschließlich der Asset-Bibliothek, nutzen.</t>
+          <t>Wenn diese Option aktiviert ist, können Hosts und Gäste speicherbezogene Funktionen, einschließlich der Asset-Bibliothek, nutzen.</t>
         </is>
       </c>
     </row>
@@ -6934,7 +6934,7 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>Tutti gli ospiti</t>
+          <t>Tutti gli host</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Inserisca l'indirizzo e-mail associato al suo conto$t(avatour)@ e la password temporanea ricevuta
+          <t>Inserisca l'indirizzo e-mail associato al suo conto$t(avatour) e la password temporanea ricevuta
  e la password temporanea che ha ricevuto, quindi
  scegliere e confermare una nuova password. La sua password deve
  essere di 8 caratteri e contenere lettere maiuscole e minuscole e numeri.</t>
@@ -8181,7 +8181,7 @@
       <c r="C351" s="4" t="inlineStr">
         <is>
           <t>&lt;1&gt;Are you sure you want to reset the password for {{email}}?&lt;/1&gt; &lt;1&gt;This will disable their current password and send them an email
-with instructions for setting a new password.&lt;/1&gt;@
+with instructions for setting a new password.&lt;/1&gt;
  &lt;1&gt;Note: Password reset email links expire after 24 hours.&lt;/1&gt;</t>
         </is>
       </c>
@@ -8276,7 +8276,7 @@
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>Inserisca l'indirizzo e-mail associato al suo$t(avatour)@ account e riceverà un link per reimpostare la password
+          <t>Inserisca l'indirizzo e-mail associato al suo$t(avatour) account e riceverà un link per reimpostare la password
  e riceverà un link per reimpostare la password.</t>
         </is>
       </c>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Oops! Qualcosa è andato storto durante il tentativo di reimpostare la sua password. Riprovi più tardi o si rivolga a &lt;0&gt;support@avatour.live&lt;/0&gt; per ricevere assistenza.</t>
+          <t>Oops! Qualcosa è andato storto durante il tentativo di reimpostare la sua password. Riprovi più tardi o si rivolga a &lt;0&gt;supportavatour.live&lt;/0&gt; per ricevere assistenza.</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -8674,7 +8674,7 @@
       </c>
       <c r="C373" s="4" t="inlineStr">
         <is>
-          <t>Per cambiare il suo dominio, contatti &lt;0&gt;support@avatour.live&lt;/0&gt;@</t>
+          <t>Per cambiare il suo dominio, contatti &lt;0&gt;supportavatour.live&lt;/0&gt;</t>
         </is>
       </c>
       <c r="D373" s="4" t="inlineStr">
@@ -8696,7 +8696,7 @@
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Non ha domini personalizzati. Contatti &lt;0&gt;support@avatour.live&lt;/0&gt; per richiedere un nuovo dominio personalizzato.</t>
+          <t>Non ha domini personalizzati. Contatti &lt;0&gt;supportavatour.live&lt;/0&gt; per richiedere un nuovo dominio personalizzato.</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -9312,7 +9312,7 @@
       </c>
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>In attesa che l'host inizi la riunione...</t>
+          <t>In attesa che Host inizi la riunione...</t>
         </is>
       </c>
       <c r="D402" s="3" t="inlineStr">
@@ -10701,7 +10701,7 @@
       </c>
       <c r="C465" s="4" t="inlineStr">
         <is>
-          <t>Sulla base dei &lt;1&gt;{{participantsUsed}}&lt;/1&gt; partecipanti con ubicazione nota, tutte le riunioni combinate hanno evitato un totale di &lt;3&gt;{{miles}} miles&lt;/3&gt;@ di viaggi aerei.</t>
+          <t>Sulla base dei &lt;1&gt;{{participantsUsed}}&lt;/1&gt; partecipanti con ubicazione nota, tutte le riunioni combinate hanno evitato un totale di &lt;3&gt;{{miles}} miles&lt;/3&gt; di viaggi aerei.</t>
         </is>
       </c>
       <c r="D465" s="4" t="inlineStr">

</xml_diff>